<commit_message>
docs: bump version to V5.1, update README, CHANGELOG, and suivi xlsx
- app.R: V5.0.0 -> V5.1 "Le Petit Prince s'envole"
- CHANGELOG: add V5.1 section (navbarPage, Home redesign, CSS cleanup)
- README: update version, module list (add mod_home, mod_sse_validation,
  helpers_ui), features table to match navbarPage layout, 175 tests
- suivi xlsx: add V5.0.0 + V5.1 rows to Changelog App, update App
  Shiny Code task, bump Dashboard date to 13/04/2026
</commit_message>
<xml_diff>
--- a/docs/suivi/suivi_projets_v2.xlsx
+++ b/docs/suivi/suivi_projets_v2.xlsx
@@ -886,7 +886,7 @@
     <row r="2" ht="18" customHeight="1" s="45">
       <c r="A2" s="47" t="inlineStr">
         <is>
-          <t>Mis à jour le 10/04/2026</t>
+          <t>Mis à jour le 13/04/2026</t>
         </is>
       </c>
     </row>
@@ -2207,120 +2207,120 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="44" t="inlineStr">
         <is>
           <t>2026-04-07</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="44" t="inlineStr">
         <is>
           <t>Frexa - Science</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="44" t="inlineStr">
         <is>
           <t>SSE validation 24 configs FIM vs empirique</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" s="44" t="inlineStr">
         <is>
           <t>Terminé</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E18" s="44" t="inlineStr">
         <is>
           <t>Basse</t>
         </is>
       </c>
-      <c r="F18" t="n">
+      <c r="F18" s="44" t="n">
         <v>100</v>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="G18" s="44" t="inlineStr">
         <is>
           <t>24 configs factorielles (3 APPROX x 4 FIMTYPE x 2 VARCROSS) comparees au SSE (200 reps PsN, 155 OK) /// FOCEI+FT1+VC0 = meilleure (79%, 11/14) /// FIMTYPE=2 = a proscrire (36-57%) /// VARCROSS depend forme variance, pas juste erreur combinee</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
+      <c r="I18" s="44" t="inlineStr">
         <is>
           <t>resultat integre dans recommandation stage</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="44" t="inlineStr">
         <is>
           <t>2026-04-03</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="44" t="inlineStr">
         <is>
           <t>Frexa - BAY0130</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C19" s="44" t="inlineStr">
         <is>
           <t>Dataset SoA frexalimab (2 bras SC/IV)</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" s="44" t="inlineStr">
         <is>
           <t>Terminé</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E19" s="44" t="inlineStr">
         <is>
           <t>Basse</t>
         </is>
       </c>
-      <c r="F19" t="n">
+      <c r="F19" s="44" t="n">
         <v>100</v>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="G19" s="44" t="inlineStr">
         <is>
           <t>dataset corrige : ISC ajoute, 2 bras (8 doses SC + 7 doses IV), 80 patients (GROUPSIZE=40) /// TSTRAT separes par voie, TMIN/TMAX a definir depuis CTP</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="I19" s="44" t="inlineStr">
         <is>
           <t>utiliser pour runs optimisation MAXEVAL&gt;0</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="44" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="44" t="inlineStr">
         <is>
           <t>Congres junior</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="44" t="inlineStr">
         <is>
           <t>Preparer slides congres 28 mai (5 slides)</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" s="44" t="inlineStr">
         <is>
           <t>En cours</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E20" s="44" t="inlineStr">
         <is>
           <t>Haute</t>
         </is>
       </c>
-      <c r="F20" t="n">
+      <c r="F20" s="44" t="n">
         <v>60</v>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="G20" s="44" t="inlineStr">
         <is>
           <t>pptx cree avec resultats FIM frexalimab, SSE validation, guide $DESIGN</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
+      <c r="I20" s="44" t="inlineStr">
         <is>
           <t>finaliser avec feedback Elisa</t>
         </is>
@@ -2506,12 +2506,12 @@
       </c>
       <c r="C5" s="71" t="inlineStr">
         <is>
-          <t>App Shiny V4 post-processing $DESIGN</t>
+          <t>App Shiny V5.1 post-processing $DESIGN</t>
         </is>
       </c>
       <c r="D5" s="71" t="inlineStr">
         <is>
-          <t>Terminé</t>
+          <t>V5.1 sur main (commit 3de476e) /// V4 -&gt; V5.0 (Home page, kill drawer, English labels) -&gt; V5.1 (navbarPage, Home redesign, CSS cleanup) /// 14 modules, 175 tests unitaires /// Power/NSN Wald + TOST equivalence, convergence steps, scatter FIM vs SSE /// compatible RStudio Server R 4.2.0</t>
         </is>
       </c>
       <c r="E5" s="71" t="inlineStr">
@@ -2524,171 +2524,171 @@
       </c>
       <c r="G5" s="71" t="inlineStr">
         <is>
-          <t>V4.5.2 sur main (PR #41 mergee) /// 14 modules (ajout SSE validation), 175 tests unitaires /// Power/NSN Wald + TOST equivalence, convergence steps, scatter FIM vs SSE /// 6 slots, pagination supprimee, launch.browser=TRUE (fix RStudio) /// refactor : split parse_design_outputs.R en 5 fichiers (&lt;425 lignes chacun) /// compatible RStudio Server R 4.2.0</t>
+          <t>V5.1 sur main /// navbarPage migration, Home two-column layout, Compare integre, settings_bar dans mod_times/mod_power, detect_method() /// refonte V5.0 : Home landing page, kill drawer, English labels, rename DE$IGN EXPLORER</t>
         </is>
       </c>
       <c r="H5" s="71" t="n"/>
       <c r="I5" s="71" t="inlineStr">
         <is>
-          <t>stabiliser sur serveur Sanofi ; refonte UI (brainstorm) ; V5 editeur .ctl</t>
+          <t>stabiliser sur serveur Sanofi ; V6 editeur .ctl</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="44" t="inlineStr">
         <is>
           <t>2026-04-07</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="44" t="inlineStr">
         <is>
           <t>App Shiny</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="44" t="inlineStr">
         <is>
           <t>V4.4.0 - Power / NSN (Wald)</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="44" t="inlineStr">
         <is>
           <t>Terminé</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="44" t="inlineStr">
         <is>
           <t>Basse</t>
         </is>
       </c>
-      <c r="F6" t="n">
+      <c r="F6" s="44" t="n">
         <v>100</v>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G6" s="44" t="inlineStr">
         <is>
           <t>module Power/NSN : compute_power_wald(), compute_n_needed(), plot_power_curve() /// tab Puissance (colore vert/orange/rouge) + tab NSN avec courbe Power(N) /// parse_groupsize() auto-rempli depuis .ctl /// 28 nouveaux tests (151 total)</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I6" s="44" t="inlineStr">
         <is>
           <t>fait - PR #37</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="44" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="44" t="inlineStr">
         <is>
           <t>App Shiny</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="44" t="inlineStr">
         <is>
           <t>V4.5.0 - TOST equivalence</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="44" t="inlineStr">
         <is>
           <t>Terminé</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="44" t="inlineStr">
         <is>
           <t>Basse</t>
         </is>
       </c>
-      <c r="F7" t="n">
+      <c r="F7" s="44" t="n">
         <v>100</v>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G7" s="44" t="inlineStr">
         <is>
           <t>test TOST (PFIM eq. 4-7) : compute_power_tost(), compute_nsn_tost() /// tab Equivalence (TOST) avec detection hors-marge, courbe Power(N) violette /// N total editable dans Power tab + encadres explicatifs Wald/TOST /// 17 nouveaux tests (175 total)</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I7" s="44" t="inlineStr">
         <is>
           <t>fait - PR #38</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="44" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="44" t="inlineStr">
         <is>
           <t>App Shiny</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="44" t="inlineStr">
         <is>
           <t>Refactor split parse_design_outputs.R</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="44" t="inlineStr">
         <is>
           <t>Terminé</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E8" s="44" t="inlineStr">
         <is>
           <t>Basse</t>
         </is>
       </c>
-      <c r="F8" t="n">
+      <c r="F8" s="44" t="n">
         <v>100</v>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G8" s="44" t="inlineStr">
         <is>
           <t>split 1268 lignes / 34 fonctions en 5 fichiers : design_utils, design_io, design_metrics, design_summary, ctl_parsers /// max 425 lignes, 0 changement API</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="I8" s="44" t="inlineStr">
         <is>
           <t>fait - PR #39</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="44" t="inlineStr">
         <is>
           <t>2026-04-10</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="44" t="inlineStr">
         <is>
           <t>App Shiny</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="44" t="inlineStr">
         <is>
           <t>V4.5.2 - SSE validation + convergence steps</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="44" t="inlineStr">
         <is>
           <t>Terminé</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E9" s="44" t="inlineStr">
         <is>
           <t>Basse</t>
         </is>
       </c>
-      <c r="F9" t="n">
+      <c r="F9" s="44" t="n">
         <v>100</v>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="G9" s="44" t="inlineStr">
         <is>
           <t>module SSE Validation (scatter FIM vs SSE, CI 95%, D-criterion, methodologie Fayette 2025) /// convergence steps (detection RS/STGR/NELDER, step chart par phase) /// PK timeline : hard cap 4 facettes, toggle h/j /// fix launch.browser=TRUE (bug RStudio viewer)</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="I9" s="44" t="inlineStr">
         <is>
           <t>fait - PR #41 + commits directs</t>
         </is>
@@ -3128,7 +3128,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="44" min="1" max="1"/>
@@ -3786,162 +3786,226 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="44" t="inlineStr">
         <is>
           <t>2026-04-07</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="44" t="inlineStr">
         <is>
           <t>V4.4.0</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="44" t="inlineStr">
         <is>
           <t>Majeure</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" s="44" t="inlineStr">
         <is>
           <t>Module Power/NSN</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E22" s="44" t="inlineStr">
         <is>
           <t>Puissance Wald + NSN par scaling FIM. Formules PopED portees. parse_groupsize() auto-rempli.</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="F22" s="44" t="inlineStr">
         <is>
           <t>PR #37</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="44" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="44" t="inlineStr">
         <is>
           <t>V4.5.0</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="44" t="inlineStr">
         <is>
           <t>Majeure</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" s="44" t="inlineStr">
         <is>
           <t>Module Power/NSN</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E23" s="44" t="inlineStr">
         <is>
           <t>TOST equivalence (PFIM eq. 4-7). N total editable. Encadres explicatifs Wald/TOST.</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="F23" s="44" t="inlineStr">
         <is>
           <t>PR #38</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="44" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="44" t="inlineStr">
         <is>
           <t>V4.5.0b</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="44" t="inlineStr">
         <is>
           <t>Refacto</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D24" s="44" t="inlineStr">
         <is>
           <t>Parsers R</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E24" s="44" t="inlineStr">
         <is>
           <t>Split parse_design_outputs.R en 5 fichiers (&lt;425 lignes). 0 changement API.</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="F24" s="44" t="inlineStr">
         <is>
           <t>PR #39</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="44" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="44" t="inlineStr">
         <is>
           <t>V4.5.1</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" s="44" t="inlineStr">
         <is>
           <t>Fix</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25" s="44" t="inlineStr">
         <is>
           <t>Module times</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="E25" s="44" t="inlineStr">
         <is>
           <t>Elementary designs (GROUPSIZE&gt;1) : detection bras par signature TSTRAT, 180-&gt;2 facettes.</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
+      <c r="F25" s="44" t="inlineStr">
         <is>
           <t>PR #40</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="44" t="inlineStr">
         <is>
           <t>2026-04-10</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="44" t="inlineStr">
         <is>
           <t>V4.5.2</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="44" t="inlineStr">
         <is>
           <t>Majeure</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" s="44" t="inlineStr">
         <is>
           <t>Module SSE + convergence</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="E26" s="44" t="inlineStr">
         <is>
           <t>SSE validation (scatter FIM vs SSE, CI 95%, D-crit). Convergence steps (RS/STGR/NELDER). PK timeline cap 4 facettes. Fix launch.browser.</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="F26" s="44" t="inlineStr">
         <is>
           <t>PR #41 + commits</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="44" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B27" s="44" t="inlineStr">
+        <is>
+          <t>V5.0.0</t>
+        </is>
+      </c>
+      <c r="C27" s="44" t="inlineStr">
+        <is>
+          <t>Majeure</t>
+        </is>
+      </c>
+      <c r="D27" s="44" t="inlineStr">
+        <is>
+          <t>App globale</t>
+        </is>
+      </c>
+      <c r="E27" s="44" t="inlineStr">
+        <is>
+          <t>Refonte V5 : Home landing page, kill drawer, English labels, rename DE$IGN EXPLORER. Upload+Examples dans Home tab.</t>
+        </is>
+      </c>
+      <c r="F27" s="44" t="inlineStr">
+        <is>
+          <t>commit 9ef08fe</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="44" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B28" s="44" t="inlineStr">
+        <is>
+          <t>V5.1</t>
+        </is>
+      </c>
+      <c r="C28" s="44" t="inlineStr">
+        <is>
+          <t>Majeure</t>
+        </is>
+      </c>
+      <c r="D28" s="44" t="inlineStr">
+        <is>
+          <t>App globale</t>
+        </is>
+      </c>
+      <c r="E28" s="44" t="inlineStr">
+        <is>
+          <t>navbarPage migration (kill conditionalPanel+JS), Home two-column layout, Compare integre dans Home, settings_bar dans mod_times/mod_power, detect_method(), CSS cleanup.</t>
+        </is>
+      </c>
+      <c r="F28" s="44" t="inlineStr">
+        <is>
+          <t>commit 3de476e</t>
         </is>
       </c>
     </row>

</xml_diff>